<commit_message>
feat: integrate Royal canonical URLs, 33 Torob links, Top 5 seller logic, and compact zero-scroll table UI
</commit_message>
<xml_diff>
--- a/data/گزارش_انبار_قیمت_به_روز.xlsx
+++ b/data/گزارش_انبار_قیمت_به_روز.xlsx
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>10950000</v>
+        <v>11390000</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>9200000</v>
@@ -664,11 +664,11 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>+1,550,000 ت از رتبه 3 ترب (+16.5%)</t>
+          <t>+1,990,000 ت از رتبه 3 ترب (+21.2%)</t>
         </is>
       </c>
       <c r="O2" s="6" t="n">
-        <v>2069550000</v>
+        <v>2141320000</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         <v>63</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>20580000</v>
+        <v>20430000</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>14590000</v>
@@ -740,15 +740,15 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>+5,081,000 ت از رتبه 3 ترب (+32.8%)</t>
+          <t>+4,931,000 ت از رتبه 3 ترب (+31.8%)</t>
         </is>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1296540000</v>
+        <v>1287090000</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1834</t>
+          <t>https://royaldigi.ir/product/netbox-mobo-edition/</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
         <v>30</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>16680000</v>
+        <v>16750000</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>12899000</v>
@@ -816,15 +816,15 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>+3,690,000 ت از رتبه 3 ترب (+28.4%)</t>
+          <t>+3,760,000 ت از رتبه 3 ترب (+28.9%)</t>
         </is>
       </c>
       <c r="O4" s="6" t="n">
-        <v>500400000</v>
+        <v>502500000</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1828</t>
+          <t>https://royaldigi.ir/product/netbox-shine-s/</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -858,10 +858,10 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>6370000</v>
+        <v>6150000</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>4500000</v>
@@ -892,11 +892,11 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>+1,370,000 ت از رتبه 3 ترب (+27.4%)</t>
+          <t>+1,150,000 ت از رتبه 3 ترب (+23.0%)</t>
         </is>
       </c>
       <c r="O5" s="6" t="n">
-        <v>114660000</v>
+        <v>104550000</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>15</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>4465000</v>
+        <v>4640000</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>3900000</v>
@@ -1044,11 +1044,11 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>+470,000 ت از رتبه 3 ترب (+11.8%)</t>
+          <t>+645,000 ت از رتبه 3 ترب (+16.1%)</t>
         </is>
       </c>
       <c r="O7" s="6" t="n">
-        <v>66975000</v>
+        <v>69600000</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -1250,10 +1250,10 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>9795000</v>
+        <v>9798000</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>8900000</v>
@@ -1284,11 +1284,11 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>+295,000 ت از رتبه 3 ترب (+3.1%)</t>
+          <t>+298,000 ت از رتبه 3 ترب (+3.1%)</t>
         </is>
       </c>
       <c r="O10" s="6" t="n">
-        <v>107745000</v>
+        <v>97980000</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1326,10 +1326,10 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>7750000</v>
+        <v>7760000</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>5900000</v>
@@ -1364,11 +1364,11 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>+1,850,000 ت از رتبه 1 ترب (+31.4%)</t>
+          <t>+1,860,000 ت از رتبه 1 ترب (+31.5%)</t>
         </is>
       </c>
       <c r="O11" s="6" t="n">
-        <v>85250000</v>
+        <v>15520000</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -1634,10 +1634,10 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>8470000</v>
+        <v>7930000</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>6200000</v>
@@ -1668,11 +1668,11 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>+2,170,000 ت از رتبه 3 ترب (+34.4%)</t>
+          <t>+1,630,000 ت از رتبه 3 ترب (+25.9%)</t>
         </is>
       </c>
       <c r="O15" s="6" t="n">
-        <v>59290000</v>
+        <v>39650000</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1964</t>
+          <t>https://royaldigi.ir/product/alcatel-bt71/</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1840</t>
+          <t>https://royaldigi.ir/product/netbox-prime/</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>9795000</v>
+        <v>9798000</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>8900000</v>
@@ -1986,15 +1986,15 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>+295,000 ت از رتبه 3 ترب (+3.1%)</t>
+          <t>+298,000 ت از رتبه 3 ترب (+3.1%)</t>
         </is>
       </c>
       <c r="O19" s="6" t="n">
-        <v>58770000</v>
+        <v>97980000</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1814</t>
+          <t>https://royaldigi.ir/product/irancell-tf-i60-s1/</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2559</t>
+          <t>https://royaldigi.ir/product/irancell-fd-m40-g1/</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1714</t>
+          <t>https://royaldigi.ir/product/tp-link-archer-c50/</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -2735,7 +2735,7 @@
         <v>4</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>5250000</v>
+        <v>5380000</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>4950000</v>
@@ -2766,11 +2766,11 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>+250,000 ت از رتبه 3 ترب (+5.0%)</t>
+          <t>+380,000 ت از رتبه 3 ترب (+7.6%)</t>
         </is>
       </c>
       <c r="O29" s="6" t="n">
-        <v>21000000</v>
+        <v>21520000</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3238</t>
+          <t>https://royaldigi.ir/product/cp108-n3004g-lte-cpe/</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
         <v>3</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>7060000</v>
+        <v>7140000</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>9600000</v>
@@ -3082,11 +3082,11 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>-2,540,000 ت از کف ترب (-26.5%)</t>
+          <t>-2,460,000 ت از کف ترب (-25.6%)</t>
         </is>
       </c>
       <c r="O33" s="6" t="n">
-        <v>21180000</v>
+        <v>21420000</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1930</t>
+          <t>https://royaldigi.ir/product/d-link-dwr-981/</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -3268,10 +3268,10 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>8820000</v>
+        <v>10100000</v>
       </c>
       <c r="G36" s="6" t="n">
         <v>6500000</v>
@@ -3302,15 +3302,15 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>+1,820,000 ت از رتبه 3 ترب (+26.0%)</t>
+          <t>+3,100,000 ت از رتبه 3 ترب (+44.3%)</t>
         </is>
       </c>
       <c r="O36" s="6" t="n">
-        <v>26460000</v>
+        <v>20200000</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1958</t>
+          <t>https://royaldigi.ir/product/utel-l443/</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
@@ -3344,10 +3344,10 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>8820000</v>
+        <v>10100000</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>6500000</v>
@@ -3378,15 +3378,15 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>+1,820,000 ت از رتبه 3 ترب (+26.0%)</t>
+          <t>+3,100,000 ت از رتبه 3 ترب (+44.3%)</t>
         </is>
       </c>
       <c r="O37" s="6" t="n">
-        <v>26460000</v>
+        <v>20200000</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1958</t>
+          <t>https://royaldigi.ir/product/utel-l443/</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
@@ -3420,10 +3420,10 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>17720000</v>
+        <v>17730000</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>11880000</v>
@@ -3456,15 +3456,15 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>+4,520,000 ت از رتبه 3 ترب (+34.2%)</t>
+          <t>+4,530,000 ت از رتبه 3 ترب (+34.3%)</t>
         </is>
       </c>
       <c r="O38" s="6" t="n">
-        <v>53160000</v>
+        <v>35460000</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2013</t>
+          <t>https://royaldigi.ir/product/irancell-tf-i60-g1/</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -3498,10 +3498,10 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>4465000</v>
+        <v>4640000</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>3900000</v>
@@ -3532,15 +3532,15 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>+470,000 ت از رتبه 3 ترب (+11.8%)</t>
+          <t>+645,000 ت از رتبه 3 ترب (+16.1%)</t>
         </is>
       </c>
       <c r="O39" s="6" t="n">
-        <v>13395000</v>
+        <v>69600000</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1753</t>
+          <t>https://royaldigi.ir/product/d-link-dsl-124/</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
@@ -3623,7 +3623,11 @@
           <t>https://royaldigi.ir/product/huawei-e5785-330-mobile-wifi-elite-2/</t>
         </is>
       </c>
-      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/8d1a9fa5-d864-4570-878e-374382235a85/%D9%85%D9%88%D8%AF%D9%85-%D9%87%D9%88%D8%A7%D9%88%DB%8C-%D9%85%D8%AF%D9%84-e5785-330/</t>
+        </is>
+      </c>
       <c r="R40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
@@ -3977,7 +3981,7 @@
         <v>2</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>7611000</v>
+        <v>7615000</v>
       </c>
       <c r="G45" s="6" t="n">
         <v>7000000</v>
@@ -4010,11 +4014,11 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>+4,000 ت از رتبه 3 ترب (+0.1%)</t>
+          <t>+8,000 ت از رتبه 3 ترب (+0.1%)</t>
         </is>
       </c>
       <c r="O45" s="6" t="n">
-        <v>15222000</v>
+        <v>15230000</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
@@ -4203,7 +4207,7 @@
         <v>2</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>9940000</v>
+        <v>12700000</v>
       </c>
       <c r="G48" s="6" t="n">
         <v>8700000</v>
@@ -4234,11 +4238,11 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>+840,000 ت از رتبه 3 ترب (+9.2%)</t>
+          <t>+3,600,000 ت از رتبه 3 ترب (+39.6%)</t>
         </is>
       </c>
       <c r="O48" s="6" t="n">
-        <v>19880000</v>
+        <v>25400000</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
@@ -4276,10 +4280,10 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>3840000</v>
+        <v>4395000</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>3140000</v>
@@ -4310,11 +4314,11 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>+690,000 ت از رتبه 3 ترب (+21.9%)</t>
+          <t>+1,245,000 ت از رتبه 3 ترب (+39.5%)</t>
         </is>
       </c>
       <c r="O49" s="6" t="n">
-        <v>7680000</v>
+        <v>4395000</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
@@ -4433,7 +4437,7 @@
         <v>2</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>17720000</v>
+        <v>17730000</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>11890000</v>
@@ -4466,11 +4470,11 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>+4,820,000 ت از رتبه 3 ترب (+37.4%)</t>
+          <t>+4,830,000 ت از رتبه 3 ترب (+37.4%)</t>
         </is>
       </c>
       <c r="O51" s="6" t="n">
-        <v>35440000</v>
+        <v>35460000</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
@@ -4589,7 +4593,7 @@
         <v>2</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>10500000</v>
+        <v>11250000</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>6750000</v>
@@ -4620,11 +4624,11 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>+3,011,000 ت از رتبه 3 ترب (+40.2%)</t>
+          <t>+3,761,000 ت از رتبه 3 ترب (+50.2%)</t>
         </is>
       </c>
       <c r="O53" s="6" t="n">
-        <v>21000000</v>
+        <v>22500000</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4748,7 +4752,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F55" s="5" t="n">
         <v>11000000</v>
@@ -4786,7 +4790,7 @@
         </is>
       </c>
       <c r="O55" s="6" t="n">
-        <v>22000000</v>
+        <v>33000000</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4827,7 +4831,7 @@
         <v>2</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>10290000</v>
+        <v>10390000</v>
       </c>
       <c r="G56" s="6" t="n">
         <v>5800000</v>
@@ -4860,11 +4864,11 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>+4,340,000 ت از رتبه 3 ترب (+72.9%)</t>
+          <t>+4,440,000 ت از رتبه 3 ترب (+74.6%)</t>
         </is>
       </c>
       <c r="O56" s="6" t="n">
-        <v>20580000</v>
+        <v>20780000</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -5256,7 +5260,7 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3231</t>
+          <t>https://royaldigi.ir/product/d-link-dwr-m961v/</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr">
@@ -5334,7 +5338,7 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2092</t>
+          <t>https://royaldigi.ir/product/tp-link-td-w8961n/</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
@@ -5448,10 +5452,10 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>5250000</v>
+        <v>5380000</v>
       </c>
       <c r="G64" s="6" t="n">
         <v>4600000</v>
@@ -5482,15 +5486,15 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>+300,000 ت از رتبه 3 ترب (+6.1%)</t>
+          <t>+430,000 ت از رتبه 3 ترب (+8.7%)</t>
         </is>
       </c>
       <c r="O64" s="6" t="n">
-        <v>10500000</v>
+        <v>21520000</v>
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1819</t>
+          <t>https://royaldigi.ir/product/irancell-fd-i40-b2/</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -5802,7 +5806,7 @@
       </c>
       <c r="P68" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3240</t>
+          <t>https://royaldigi.ir/product/huawei-echolife-hg8546m/</t>
         </is>
       </c>
       <c r="Q68" s="2" t="inlineStr">
@@ -5916,7 +5920,7 @@
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" s="5" t="n">
         <v>9550000</v>
@@ -5960,11 +5964,11 @@
         </is>
       </c>
       <c r="O70" s="6" t="n">
-        <v>19100000</v>
+        <v>9550000</v>
       </c>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1885</t>
+          <t>https://royaldigi.ir/product/huawei-e5577c/</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
@@ -6126,7 +6130,7 @@
       </c>
       <c r="P72" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1914</t>
+          <t>https://royaldigi.ir/product/huawei-e5783-330/</t>
         </is>
       </c>
       <c r="Q72" s="2" t="inlineStr">
@@ -6160,10 +6164,10 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>4460000</v>
+        <v>4475000</v>
       </c>
       <c r="G73" s="6" t="n">
         <v>3290000</v>
@@ -6194,15 +6198,15 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>+570,000 ت از رتبه 3 ترب (+14.7%)</t>
+          <t>+585,000 ت از رتبه 3 ترب (+15.0%)</t>
         </is>
       </c>
       <c r="O73" s="6" t="n">
-        <v>8920000</v>
+        <v>4475000</v>
       </c>
       <c r="P73" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2127</t>
+          <t>https://royaldigi.ir/product/vodafone-r228t/</t>
         </is>
       </c>
       <c r="Q73" s="2" t="inlineStr">
@@ -6239,7 +6243,7 @@
         <v>1</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>12010000</v>
+        <v>12005000</v>
       </c>
       <c r="G74" s="6" t="n">
         <v>8999000</v>
@@ -6270,15 +6274,15 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>+2,810,000 ت از رتبه 3 ترب (+30.5%)</t>
+          <t>+2,805,000 ت از رتبه 3 ترب (+30.5%)</t>
         </is>
       </c>
       <c r="O74" s="6" t="n">
-        <v>12010000</v>
+        <v>12005000</v>
       </c>
       <c r="P74" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2553</t>
+          <t>https://royaldigi.ir/product/tp-link-tl-wa901n/</t>
         </is>
       </c>
       <c r="Q74" s="2" t="inlineStr">
@@ -6315,7 +6319,7 @@
         <v>1</v>
       </c>
       <c r="F75" s="5" t="n">
-        <v>22000000</v>
+        <v>21740000</v>
       </c>
       <c r="G75" s="6" t="n">
         <v>2350000</v>
@@ -6346,15 +6350,15 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>+19,555,000 ت از رتبه 3 ترب (+799.8%)</t>
+          <t>+19,295,000 ت از رتبه 3 ترب (+789.2%)</t>
         </is>
       </c>
       <c r="O75" s="6" t="n">
-        <v>22000000</v>
+        <v>21740000</v>
       </c>
       <c r="P75" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2552</t>
+          <t>https://royaldigi.ir/product/tp-link-eap225-v3/</t>
         </is>
       </c>
       <c r="Q75" s="2" t="inlineStr">
@@ -6387,7 +6391,7 @@
         <v>1</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>27470000</v>
+        <v>27370000</v>
       </c>
       <c r="G76" s="6" t="n">
         <v>10000000</v>
@@ -6418,15 +6422,15 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>+11,870,000 ت از رتبه 3 ترب (+76.1%)</t>
+          <t>+11,770,000 ت از رتبه 3 ترب (+75.4%)</t>
         </is>
       </c>
       <c r="O76" s="6" t="n">
-        <v>27470000</v>
+        <v>27370000</v>
       </c>
       <c r="P76" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3229</t>
+          <t>https://royaldigi.ir/product/tp-link-omada-eap245-v3/</t>
         </is>
       </c>
       <c r="Q76" s="2" t="inlineStr">
@@ -6459,7 +6463,7 @@
         <v>1</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>9990000</v>
+        <v>10740000</v>
       </c>
       <c r="G77" s="6" t="n">
         <v>8999000</v>
@@ -6490,15 +6494,15 @@
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>+790,000 ت از رتبه 3 ترب (+8.6%)</t>
+          <t>+1,540,000 ت از رتبه 3 ترب (+16.7%)</t>
         </is>
       </c>
       <c r="O77" s="6" t="n">
-        <v>9990000</v>
+        <v>10740000</v>
       </c>
       <c r="P77" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2551</t>
+          <t>https://royaldigi.ir/product/tp-link-eap110-outdoor/</t>
         </is>
       </c>
       <c r="Q77" s="2" t="inlineStr">
@@ -6611,7 +6615,7 @@
         <v>1</v>
       </c>
       <c r="F79" s="5" t="n">
-        <v>4950000</v>
+        <v>4540000</v>
       </c>
       <c r="G79" s="6" t="n">
         <v>3750000</v>
@@ -6642,15 +6646,15 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>+1,095,000 ت از رتبه 3 ترب (+28.4%)</t>
+          <t>+685,000 ت از رتبه 3 ترب (+17.8%)</t>
         </is>
       </c>
       <c r="O79" s="6" t="n">
-        <v>4950000</v>
+        <v>4540000</v>
       </c>
       <c r="P79" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2554</t>
+          <t>https://royaldigi.ir/product/tp-link-tl-wr840n/</t>
         </is>
       </c>
       <c r="Q79" s="2" t="inlineStr">
@@ -6687,7 +6691,7 @@
         <v>1</v>
       </c>
       <c r="F80" s="5" t="n">
-        <v>15495000</v>
+        <v>15498000</v>
       </c>
       <c r="G80" s="6" t="n">
         <v>14700000</v>
@@ -6718,11 +6722,11 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>+505,000 ت از رتبه 3 ترب (+3.4%)</t>
+          <t>+508,000 ت از رتبه 3 ترب (+3.4%)</t>
         </is>
       </c>
       <c r="O80" s="6" t="n">
-        <v>15495000</v>
+        <v>15498000</v>
       </c>
       <c r="P80" s="2" t="inlineStr">
         <is>
@@ -6763,7 +6767,7 @@
         <v>1</v>
       </c>
       <c r="F81" s="5" t="n">
-        <v>6495000</v>
+        <v>6500000</v>
       </c>
       <c r="G81" s="6" t="n">
         <v>6190000</v>
@@ -6794,15 +6798,15 @@
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>+295,000 ت از رتبه 3 ترب (+4.8%)</t>
+          <t>+300,000 ت از رتبه 3 ترب (+4.8%)</t>
         </is>
       </c>
       <c r="O81" s="6" t="n">
-        <v>6495000</v>
+        <v>6500000</v>
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2555</t>
+          <t>https://royaldigi.ir/product/tp-link-archer-c6/</t>
         </is>
       </c>
       <c r="Q81" s="2" t="inlineStr">
@@ -6917,7 +6921,7 @@
         <v>1</v>
       </c>
       <c r="F83" s="5" t="n">
-        <v>15780000</v>
+        <v>22200000</v>
       </c>
       <c r="G83" s="6" t="n">
         <v>10000000</v>
@@ -6948,15 +6952,15 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>+3,980,000 ت از رتبه 3 ترب (+33.7%)</t>
+          <t>+10,400,000 ت از رتبه 3 ترب (+88.1%)</t>
         </is>
       </c>
       <c r="O83" s="6" t="n">
-        <v>15780000</v>
+        <v>22200000</v>
       </c>
       <c r="P83" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3245</t>
+          <t>https://royaldigi.ir/product/dlink-dir-x3000z-vodafone/</t>
         </is>
       </c>
       <c r="Q83" s="2" t="inlineStr">
@@ -6993,7 +6997,7 @@
         <v>1</v>
       </c>
       <c r="F84" s="5" t="n">
-        <v>2660000</v>
+        <v>2652000</v>
       </c>
       <c r="G84" s="6" t="n">
         <v>2350000</v>
@@ -7024,15 +7028,15 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>+215,000 ت از رتبه 3 ترب (+8.8%)</t>
+          <t>+207,000 ت از رتبه 3 ترب (+8.5%)</t>
         </is>
       </c>
       <c r="O84" s="6" t="n">
-        <v>2660000</v>
+        <v>2652000</v>
       </c>
       <c r="P84" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2556</t>
+          <t>https://royaldigi.ir/product/d-link-dgs-1005a/</t>
         </is>
       </c>
       <c r="Q84" s="2" t="inlineStr">
@@ -7104,7 +7108,7 @@
       </c>
       <c r="P85" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2568</t>
+          <t>https://royaldigi.ir/product/tp-link-re200/</t>
         </is>
       </c>
       <c r="Q85" s="2" t="inlineStr">
@@ -7190,7 +7194,7 @@
       </c>
       <c r="P86" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3243</t>
+          <t>https://royaldigi.ir/product/bvot-u20/</t>
         </is>
       </c>
       <c r="Q86" s="2" t="inlineStr">
@@ -7272,7 +7276,7 @@
       </c>
       <c r="P87" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2565</t>
+          <t>https://royaldigi.ir/product/huawei-carfi-e8377/</t>
         </is>
       </c>
       <c r="Q87" s="2" t="inlineStr">
@@ -7384,10 +7388,10 @@
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>8820000</v>
+        <v>10100000</v>
       </c>
       <c r="G89" s="6" t="n">
         <v>6400000</v>
@@ -7418,11 +7422,11 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>+1,870,000 ت از رتبه 3 ترب (+26.9%)</t>
+          <t>+3,150,000 ت از رتبه 3 ترب (+45.3%)</t>
         </is>
       </c>
       <c r="O89" s="6" t="n">
-        <v>8820000</v>
+        <v>20200000</v>
       </c>
       <c r="P89" s="2" t="inlineStr">
         <is>
@@ -7460,10 +7464,10 @@
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>8820000</v>
+        <v>10100000</v>
       </c>
       <c r="G90" s="6" t="n">
         <v>6400000</v>
@@ -7494,11 +7498,11 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>+1,870,000 ت از رتبه 3 ترب (+26.9%)</t>
+          <t>+3,150,000 ت از رتبه 3 ترب (+45.3%)</t>
         </is>
       </c>
       <c r="O90" s="6" t="n">
-        <v>8820000</v>
+        <v>20200000</v>
       </c>
       <c r="P90" s="2" t="inlineStr">
         <is>
@@ -7617,7 +7621,7 @@
         <v>1</v>
       </c>
       <c r="F92" s="5" t="n">
-        <v>3508000</v>
+        <v>3501000</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>2900000</v>
@@ -7648,11 +7652,11 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>+520,000 ت از رتبه 3 ترب (+17.4%)</t>
+          <t>+513,000 ت از رتبه 3 ترب (+17.2%)</t>
         </is>
       </c>
       <c r="O92" s="6" t="n">
-        <v>3508000</v>
+        <v>3501000</v>
       </c>
       <c r="P92" s="2" t="inlineStr">
         <is>
@@ -7693,7 +7697,7 @@
         <v>1</v>
       </c>
       <c r="F93" s="5" t="n">
-        <v>7979500</v>
+        <v>7900000</v>
       </c>
       <c r="G93" s="6" t="n">
         <v>6898000</v>
@@ -7724,15 +7728,15 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>+1,059,500 ت از رتبه 3 ترب (+15.3%)</t>
+          <t>+980,000 ت از رتبه 3 ترب (+14.2%)</t>
         </is>
       </c>
       <c r="O93" s="6" t="n">
-        <v>7979500</v>
+        <v>7900000</v>
       </c>
       <c r="P93" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2162</t>
+          <t>https://royaldigi.ir/product/utel-g442/</t>
         </is>
       </c>
       <c r="Q93" s="2" t="inlineStr">
@@ -7769,7 +7773,7 @@
         <v>1</v>
       </c>
       <c r="F94" s="9" t="n">
-        <v>5800000</v>
+        <v>5889000</v>
       </c>
       <c r="G94" s="6" t="n">
         <v>3580000</v>
@@ -7808,7 +7812,7 @@
         </is>
       </c>
       <c r="O94" s="6" t="n">
-        <v>5800000</v>
+        <v>5889000</v>
       </c>
       <c r="P94" s="2" t="inlineStr">
         <is>
@@ -7925,7 +7929,7 @@
         <v>1</v>
       </c>
       <c r="F96" s="5" t="n">
-        <v>5010000</v>
+        <v>5040000</v>
       </c>
       <c r="G96" s="6" t="n">
         <v>4500000</v>
@@ -7962,11 +7966,11 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>+510,000 ت از رتبه 1 ترب (+11.3%)</t>
+          <t>+540,000 ت از رتبه 1 ترب (+12.0%)</t>
         </is>
       </c>
       <c r="O96" s="6" t="n">
-        <v>5010000</v>
+        <v>5040000</v>
       </c>
       <c r="P96" s="2" t="inlineStr">
         <is>
@@ -8052,7 +8056,7 @@
       </c>
       <c r="P97" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1885</t>
+          <t>https://royaldigi.ir/product/huawei-e5577c/</t>
         </is>
       </c>
       <c r="Q97" s="2" t="inlineStr">
@@ -8086,7 +8090,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F98" s="5" t="n">
         <v>11000000</v>
@@ -8124,7 +8128,7 @@
         </is>
       </c>
       <c r="O98" s="6" t="n">
-        <v>11000000</v>
+        <v>33000000</v>
       </c>
       <c r="P98" s="2" t="inlineStr">
         <is>
@@ -8165,7 +8169,7 @@
         <v>1</v>
       </c>
       <c r="F99" s="5" t="n">
-        <v>4460000</v>
+        <v>4475000</v>
       </c>
       <c r="G99" s="6" t="n">
         <v>3290000</v>
@@ -8196,11 +8200,11 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>+570,000 ت از رتبه 3 ترب (+14.7%)</t>
+          <t>+585,000 ت از رتبه 3 ترب (+15.0%)</t>
         </is>
       </c>
       <c r="O99" s="6" t="n">
-        <v>4460000</v>
+        <v>4475000</v>
       </c>
       <c r="P99" s="2" t="inlineStr">
         <is>
@@ -8284,7 +8288,7 @@
       </c>
       <c r="P100" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1997</t>
+          <t>https://royaldigi.ir/product/irancell-dt-350/</t>
         </is>
       </c>
       <c r="Q100" s="2" t="inlineStr">
@@ -8364,10 +8368,14 @@
       </c>
       <c r="P101" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3250</t>
-        </is>
-      </c>
-      <c r="Q101" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/mikrotik-rb750r2/</t>
+        </is>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/fdd3ab52-7612-4fc0-8237-40c7fa31655e/%D8%B1%D9%88%D8%AA%D8%B1-%D9%85%DB%8C%DA%A9%D8%B1%D9%88%D8%AA%DB%8C%DA%A9-%D9%85%D8%AF%D9%84-hex-lite-_-rb750gr2/</t>
+        </is>
+      </c>
       <c r="R101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
@@ -8393,7 +8401,7 @@
         <v>1</v>
       </c>
       <c r="F102" s="9" t="n">
-        <v>27470000</v>
+        <v>27370000</v>
       </c>
       <c r="G102" s="6" t="n">
         <v>25757000</v>
@@ -8430,14 +8438,18 @@
         </is>
       </c>
       <c r="O102" s="6" t="n">
-        <v>27470000</v>
+        <v>27370000</v>
       </c>
       <c r="P102" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3229</t>
-        </is>
-      </c>
-      <c r="Q102" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/tp-link-omada-eap245-v3/</t>
+        </is>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/9207040a-f0f8-40af-b983-93881477740e/</t>
+        </is>
+      </c>
       <c r="R102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
@@ -8460,7 +8472,7 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F103" s="6" t="n">
         <v>12060000</v>
@@ -8506,11 +8518,11 @@
         </is>
       </c>
       <c r="O103" s="6" t="n">
-        <v>12060000</v>
+        <v>72360000</v>
       </c>
       <c r="P103" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1840</t>
+          <t>https://royaldigi.ir/product/netbox-prime/</t>
         </is>
       </c>
       <c r="Q103" s="2" t="inlineStr">
@@ -8547,7 +8559,7 @@
         <v>1</v>
       </c>
       <c r="F104" s="5" t="n">
-        <v>4950000</v>
+        <v>4540000</v>
       </c>
       <c r="G104" s="6" t="n">
         <v>3750000</v>
@@ -8578,15 +8590,15 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>+1,095,000 ت از رتبه 3 ترب (+28.4%)</t>
+          <t>+685,000 ت از رتبه 3 ترب (+17.8%)</t>
         </is>
       </c>
       <c r="O104" s="6" t="n">
-        <v>4950000</v>
+        <v>4540000</v>
       </c>
       <c r="P104" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2554</t>
+          <t>https://royaldigi.ir/product/tp-link-tl-wr840n/</t>
         </is>
       </c>
       <c r="Q104" s="2" t="inlineStr">
@@ -8664,7 +8676,7 @@
       </c>
       <c r="P105" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3227</t>
+          <t>https://royaldigi.ir/product/d-link-des-1008a/</t>
         </is>
       </c>
       <c r="Q105" s="2" t="inlineStr">
@@ -8744,7 +8756,7 @@
       </c>
       <c r="P106" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3232</t>
+          <t>https://royaldigi.ir/product/alcatel-linkzone-mw70vk-cat-7/</t>
         </is>
       </c>
       <c r="Q106" s="2" t="inlineStr">
@@ -8830,7 +8842,7 @@
       </c>
       <c r="P107" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3242</t>
+          <t>https://royaldigi.ir/product/jazz-mf673/</t>
         </is>
       </c>
       <c r="Q107" s="2" t="inlineStr">
@@ -8908,7 +8920,7 @@
       </c>
       <c r="P108" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1868</t>
+          <t>https://royaldigi.ir/product/tp-link-m7200/</t>
         </is>
       </c>
       <c r="Q108" s="2" t="inlineStr">
@@ -9068,7 +9080,7 @@
       </c>
       <c r="P110" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3228</t>
+          <t>https://royaldigi.ir/product/irancell-gp-2101-plus/</t>
         </is>
       </c>
       <c r="Q110" s="2" t="inlineStr">
@@ -9154,7 +9166,7 @@
       </c>
       <c r="P111" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3233</t>
+          <t>https://royaldigi.ir/product/asiacell-speedoo-huawei-e352/</t>
         </is>
       </c>
       <c r="Q111" s="2" t="inlineStr">
@@ -9240,7 +9252,7 @@
       </c>
       <c r="P112" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3251</t>
+          <t>https://royaldigi.ir/product/%d9%85%d9%88%d8%af%d9%85-%d8%b1%d9%88%d8%aa%d8%b1-4-5g-lte-%d8%af%d9%88-%d8%a8%d8%a7%d9%86%d8%af%d9%87-%d9%86%d8%b2%d8%aa%da%a9-naztech-nzt-gtx1000/</t>
         </is>
       </c>
       <c r="Q112" s="2" t="inlineStr">
@@ -9513,7 +9525,7 @@
         <v>1</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>3508000</v>
+        <v>3501000</v>
       </c>
       <c r="G116" s="6" t="n">
         <v>2900000</v>
@@ -9544,15 +9556,15 @@
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>+520,000 ت از رتبه 3 ترب (+17.4%)</t>
+          <t>+513,000 ت از رتبه 3 ترب (+17.2%)</t>
         </is>
       </c>
       <c r="O116" s="6" t="n">
-        <v>3508000</v>
+        <v>3501000</v>
       </c>
       <c r="P116" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1809</t>
+          <t>https://royaldigi.ir/product/neterbit-nsl-122/</t>
         </is>
       </c>
       <c r="Q116" s="2" t="inlineStr">
@@ -9634,7 +9646,7 @@
       </c>
       <c r="P117" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3239</t>
+          <t>https://royaldigi.ir/product/huawei-hg655d-n300/</t>
         </is>
       </c>
       <c r="Q117" s="2" t="inlineStr">
@@ -9748,10 +9760,10 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F119" s="5" t="n">
-        <v>10500000</v>
+        <v>11250000</v>
       </c>
       <c r="G119" s="6" t="n">
         <v>6750000</v>
@@ -9782,15 +9794,15 @@
       </c>
       <c r="N119" s="2" t="inlineStr">
         <is>
-          <t>+3,011,000 ت از رتبه 3 ترب (+40.2%)</t>
+          <t>+3,761,000 ت از رتبه 3 ترب (+50.2%)</t>
         </is>
       </c>
       <c r="O119" s="6" t="n">
-        <v>10500000</v>
+        <v>22500000</v>
       </c>
       <c r="P119" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2115</t>
+          <t>https://royaldigi.ir/product/d-link-dwr-m921/</t>
         </is>
       </c>
       <c r="Q119" s="2" t="inlineStr">
@@ -9870,7 +9882,7 @@
       </c>
       <c r="P120" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2563</t>
+          <t>https://royaldigi.ir/product/mobinnet-mn-4200-n/</t>
         </is>
       </c>
       <c r="Q120" s="2" t="inlineStr">
@@ -9950,7 +9962,7 @@
       </c>
       <c r="P121" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2567</t>
+          <t>https://royaldigi.ir/product/huawei-speed-wi-fi-home-l01s/</t>
         </is>
       </c>
       <c r="Q121" s="2" t="inlineStr">
@@ -10132,10 +10144,10 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F124" s="11" t="n">
-        <v>7060000</v>
+        <v>7140000</v>
       </c>
       <c r="G124" s="6" t="n">
         <v>9600000</v>
@@ -10172,15 +10184,15 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>-2,540,000 ت از کف ترب (-26.5%)</t>
+          <t>-2,460,000 ت از کف ترب (-25.6%)</t>
         </is>
       </c>
       <c r="O124" s="6" t="n">
-        <v>7060000</v>
+        <v>21420000</v>
       </c>
       <c r="P124" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1851</t>
+          <t>https://royaldigi.ir/product/tp-link-xn020-g3/</t>
         </is>
       </c>
       <c r="Q124" s="2" t="inlineStr">
@@ -10262,7 +10274,7 @@
       </c>
       <c r="P125" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3244</t>
+          <t>https://royaldigi.ir/product/zlt-x20-ooredoo/</t>
         </is>
       </c>
       <c r="Q125" s="2" t="inlineStr">
@@ -10340,7 +10352,7 @@
       </c>
       <c r="P126" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2566</t>
+          <t>https://royaldigi.ir/product/huawei-b2368/</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
@@ -10460,7 +10472,7 @@
         </is>
       </c>
       <c r="E128" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F128" s="5" t="n">
         <v>11000000</v>
@@ -10498,11 +10510,11 @@
         </is>
       </c>
       <c r="O128" s="6" t="n">
-        <v>11000000</v>
+        <v>33000000</v>
       </c>
       <c r="P128" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1879</t>
+          <t>https://royaldigi.ir/product/huawei-e5573-320/</t>
         </is>
       </c>
       <c r="Q128" s="2" t="inlineStr">
@@ -10668,7 +10680,7 @@
       </c>
       <c r="P130" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2558</t>
+          <t>https://royaldigi.ir/product/irancell-fd-m40-b1/</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
@@ -10862,7 +10874,7 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F133" s="5" t="n">
         <v>21750000</v>
@@ -10900,11 +10912,11 @@
         </is>
       </c>
       <c r="O133" s="6" t="n">
-        <v>21750000</v>
+        <v>108750000</v>
       </c>
       <c r="P133" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1770</t>
+          <t>https://royaldigi.ir/product/naztech-hope/</t>
         </is>
       </c>
       <c r="Q133" s="2" t="inlineStr">
@@ -10984,7 +10996,7 @@
       </c>
       <c r="P134" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3236</t>
+          <t>https://royaldigi.ir/product/huawei-b622-335/</t>
         </is>
       </c>
       <c r="Q134" s="2" t="inlineStr">
@@ -11070,10 +11082,14 @@
       </c>
       <c r="P135" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1975</t>
-        </is>
-      </c>
-      <c r="Q135" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/alcatel-linkzone-mw40v/</t>
+        </is>
+      </c>
+      <c r="Q135" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/698b55f2-da18-42c9-a207-63d2803d366d/%D9%85%D9%88%D8%AF%D9%85-%D8%AC%DB%8C%D8%A8%DB%8C-%D8%A7%D9%84%DA%A9%D8%A7%D8%AA%D9%84-linkzone-mw40v-4g/</t>
+        </is>
+      </c>
       <c r="R135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
@@ -11140,10 +11156,14 @@
       </c>
       <c r="P136" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1973</t>
-        </is>
-      </c>
-      <c r="Q136" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/d-link-dwr-930m/</t>
+        </is>
+      </c>
+      <c r="Q136" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3c5544f1-2704-4dcb-a918-a41d404325f8/%D9%85%D9%88%D8%AF%D9%85-4g-%D9%82%D8%A7%D8%A8%D9%84-%D8%AD%D9%85%D9%84-%D8%AF%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-%D9%85%D8%AF%D9%84-dwr-930m/</t>
+        </is>
+      </c>
       <c r="R136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
@@ -11212,10 +11232,14 @@
       </c>
       <c r="P137" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2057</t>
-        </is>
-      </c>
-      <c r="Q137" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/d-link-dwr-933v/</t>
+        </is>
+      </c>
+      <c r="Q137" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/613960de-720e-4f00-afd5-3ce32b01df80/%D9%85%D9%88%D8%AF%D9%85-%D8%B1%D9%88%D8%AA%D8%B1-%D8%A8%DB%8C-%D8%B3%DB%8C%D9%85-%D8%AF%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-%D9%85%D8%AF%D9%84-dwr-933v-4g-lte/</t>
+        </is>
+      </c>
       <c r="R137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
@@ -11282,10 +11306,14 @@
       </c>
       <c r="P138" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2076</t>
-        </is>
-      </c>
-      <c r="Q138" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/d-link-dwr-m920/</t>
+        </is>
+      </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/7b905a85-31a3-4aa4-8cb0-c623df59507d/%D9%85%D9%88%D8%AF%D9%85-%D8%AF%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-%D9%85%D8%AF%D9%84-dwr-m920/</t>
+        </is>
+      </c>
       <c r="R138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
@@ -11352,10 +11380,14 @@
       </c>
       <c r="P139" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2562</t>
-        </is>
-      </c>
-      <c r="Q139" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/huawei-du-h155-380/</t>
+        </is>
+      </c>
+      <c r="Q139" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/354d19d6-5474-4b53-9f5b-b9f05a183533/</t>
+        </is>
+      </c>
       <c r="R139" s="2" t="inlineStr"/>
     </row>
     <row r="140">
@@ -11502,10 +11534,14 @@
       </c>
       <c r="P141" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2550</t>
-        </is>
-      </c>
-      <c r="Q141" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/huawei-w435-md-500b/</t>
+        </is>
+      </c>
+      <c r="Q141" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/b5042640-6b61-4817-a0be-4907f7544b91/%D8%A7%D9%86%D8%AA%D9%86-%D8%AA%D9%82%D9%88%DB%8C%D8%AA%DB%8C-%D9%85%D9%88%D8%AF%D9%85-%D8%AC%DB%8C%D8%A8%DB%8C-%D9%85%D8%AF%D9%84-w435/</t>
+        </is>
+      </c>
       <c r="R141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
@@ -11580,10 +11616,14 @@
       </c>
       <c r="P142" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2031</t>
-        </is>
-      </c>
-      <c r="Q142" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/irancell-fd-i40-g1/</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/0531db72-7b60-4ae7-addb-bbca662a8e5f/%D9%85%D9%88%D8%AF%D9%85-%D8%B1%D9%88%D9%85%DB%8C%D8%B2%DB%8C-3g-4g-%D8%A7%DB%8C%D8%B1%D8%A7%D9%86%D8%B3%D9%84-%D9%85%D8%AF%D9%84-fd-i40-g1/</t>
+        </is>
+      </c>
       <c r="R142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
@@ -11652,10 +11692,14 @@
       </c>
       <c r="P143" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2040</t>
-        </is>
-      </c>
-      <c r="Q143" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/irancell-lh92/</t>
+        </is>
+      </c>
+      <c r="Q143" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/6891435a-41ca-47e6-b6a9-644c3e5898cf/%D9%85%D9%88%D8%AF%D9%85-%D9%87%D9%85%D8%B1%D8%A7%D9%87-%D8%A7%DB%8C%D8%B1%D8%A7%D9%86%D8%B3%D9%84-%D9%85%D8%AF%D9%84-lh92-4g/</t>
+        </is>
+      </c>
       <c r="R143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
@@ -11724,10 +11768,14 @@
       </c>
       <c r="P144" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2046</t>
-        </is>
-      </c>
-      <c r="Q144" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/irancell-lh96/</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3c985055-6674-4b5c-a5d3-f5424578c734/</t>
+        </is>
+      </c>
       <c r="R144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
@@ -11791,7 +11839,11 @@
         <v>0</v>
       </c>
       <c r="P145" s="2" t="inlineStr"/>
-      <c r="Q145" s="2" t="inlineStr"/>
+      <c r="Q145" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3f4bb37d-893b-4742-9309-51abed232a46/%D9%85%D9%88%D8%AF%D9%85-%D8%A7%DB%8C%D8%B1%D8%A7%D9%86%D8%B3%D9%84-%D9%85%D8%AF%D9%84-tf-i60-s1/</t>
+        </is>
+      </c>
       <c r="R145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
@@ -11866,7 +11918,7 @@
       </c>
       <c r="P146" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2142</t>
+          <t>https://royaldigi.ir/product/irancell-uroad-ss10/</t>
         </is>
       </c>
       <c r="Q146" s="2" t="inlineStr"/>
@@ -11938,10 +11990,14 @@
       </c>
       <c r="P147" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3247</t>
-        </is>
-      </c>
-      <c r="Q147" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/klpda18dbi-25m/</t>
+        </is>
+      </c>
+      <c r="Q147" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3b1d3d63-2b36-4c4c-83b6-2007823f990a/</t>
+        </is>
+      </c>
       <c r="R147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
@@ -12009,7 +12065,11 @@
         <v>0</v>
       </c>
       <c r="P148" s="2" t="inlineStr"/>
-      <c r="Q148" s="2" t="inlineStr"/>
+      <c r="Q148" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/653303c6-07f7-418e-a988-912f2750e386/</t>
+        </is>
+      </c>
       <c r="R148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
@@ -12078,10 +12138,14 @@
       </c>
       <c r="P149" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1932</t>
-        </is>
-      </c>
-      <c r="Q149" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/mci-ha4300/</t>
+        </is>
+      </c>
+      <c r="Q149" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/1628d055-6111-40b9-810a-3c5b8b93910c/</t>
+        </is>
+      </c>
       <c r="R149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
@@ -12156,7 +12220,7 @@
       </c>
       <c r="P150" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2557</t>
+          <t>https://royaldigi.ir/product/mp-link-mp-4844/</t>
         </is>
       </c>
       <c r="Q150" s="2" t="inlineStr"/>
@@ -12234,10 +12298,14 @@
       </c>
       <c r="P151" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2561</t>
-        </is>
-      </c>
-      <c r="Q151" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/necton-lc-02/</t>
+        </is>
+      </c>
+      <c r="Q151" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/a3154f97-1352-4361-b244-6899a5746f89/%D9%85%D9%88%D8%AF%D9%85-%D8%B1%D9%88%D9%85%DB%8C%D8%B2%DB%8C-%D9%86%DA%A9%D8%AA%D9%88%D9%86-%D9%85%D8%AF%D9%84-lc02-td-lte-45g/</t>
+        </is>
+      </c>
       <c r="R151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
@@ -12304,10 +12372,14 @@
       </c>
       <c r="P152" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1897</t>
-        </is>
-      </c>
-      <c r="Q152" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/tp-link-eap110/</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/65306660-8430-4e3a-9669-02685764d852/</t>
+        </is>
+      </c>
       <c r="R152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
@@ -12374,10 +12446,14 @@
       </c>
       <c r="P153" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2560</t>
-        </is>
-      </c>
-      <c r="Q153" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/ugalink-ug-4221/</t>
+        </is>
+      </c>
+      <c r="Q153" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/e3427f1b-3f2d-4874-a690-366551b74f07/</t>
+        </is>
+      </c>
       <c r="R153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
@@ -12444,10 +12520,14 @@
       </c>
       <c r="P154" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=1737</t>
-        </is>
-      </c>
-      <c r="Q154" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/zte-mc801a/</t>
+        </is>
+      </c>
+      <c r="Q154" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/94833b95-d250-482f-870b-53c847d17482/</t>
+        </is>
+      </c>
       <c r="R154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
@@ -12522,10 +12602,14 @@
       </c>
       <c r="P155" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3249</t>
-        </is>
-      </c>
-      <c r="Q155" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/ubiquiti-uap-ac-lr/</t>
+        </is>
+      </c>
+      <c r="Q155" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/a4773c33-652a-4340-9a28-112349195325/</t>
+        </is>
+      </c>
       <c r="R155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
@@ -12600,10 +12684,14 @@
       </c>
       <c r="P156" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3237</t>
-        </is>
-      </c>
-      <c r="Q156" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/%d8%a8%d8%a7%d8%aa%d8%b1%db%8c-%d9%85%d9%88%d8%af%d9%85-m40-g1-%d9%85%d8%af%d9%84-l816-%d8%b8%d8%b1%d9%81%db%8c%d8%aa-2100mah/</t>
+        </is>
+      </c>
+      <c r="Q156" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/8525b6a7-0130-47ec-a472-88f5a2b16624/</t>
+        </is>
+      </c>
       <c r="R156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
@@ -12681,7 +12769,11 @@
           <t>https://royaldigi.ir/product/tp-link-tl-wr941nd/</t>
         </is>
       </c>
-      <c r="Q157" s="2" t="inlineStr"/>
+      <c r="Q157" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/a46c3786-ab3d-4e09-8471-3cb415de2742/%D8%B1%D9%88%D8%AA%D8%B1-%D8%A8%DB%8C-%D8%B3%DB%8C%D9%85-%D8%AA%DA%A9-%D8%A8%D8%A7%D9%86%D8%AF%D9%87-%D8%AA%DB%8C-%D9%BE%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-tp-link-tl-wr941nd-%D8%A7%DA%A9%D8%A8%D9%86%D8%AF/</t>
+        </is>
+      </c>
       <c r="R157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
@@ -12759,7 +12851,11 @@
           <t>https://royaldigi.ir/product/tp-link-archer-ax3000/</t>
         </is>
       </c>
-      <c r="Q158" s="2" t="inlineStr"/>
+      <c r="Q158" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3e2f8716-b861-494b-900a-33da78c9db29/%D8%B1%D9%88%D8%AA%D8%B1-%D8%A8%DB%8C-%D8%B3%DB%8C%D9%85-%D8%AA%DB%8C-%D9%BE%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-%D9%85%D8%AF%D9%84-archer-ax55-%D8%B8%D8%B1%D9%81%DB%8C%D8%AA-ax3000/</t>
+        </is>
+      </c>
       <c r="R158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
@@ -12837,7 +12933,11 @@
           <t>https://royaldigi.ir/product/tp-link-archer-c60-v3/</t>
         </is>
       </c>
-      <c r="Q159" s="2" t="inlineStr"/>
+      <c r="Q159" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/5d00374d-afa7-42ac-9f67-3ccba7601c8f/%D8%B1%D9%88%D8%AA%D8%B1-%D8%A8%DB%8C-%D8%B3%DB%8C%D9%85-%D8%AA%DB%8C-%D9%BE%DB%8C-%D9%84%DB%8C%D9%86%DA%A9-archer-c60-ac1350-%D8%AF%D9%88-%D8%A8%D8%A7%D9%86%D8%AF/</t>
+        </is>
+      </c>
       <c r="R159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
@@ -12912,10 +13012,14 @@
       </c>
       <c r="P160" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=3248</t>
-        </is>
-      </c>
-      <c r="Q160" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/%da%a9%d8%a7%d8%a8%d9%84-%d9%85%d8%a8%d8%af%d9%84-%d8%a7%d9%81%d8%b2%d8%a7%db%8c%d9%86%d8%af%d9%87-%d9%88%d9%84%d8%aa%d8%a7%da%98-usb-5v-%d8%a8%d9%87-dc-12v-%d9%85%d8%ae%d8%b5%d9%88%d8%b5-%d9%85%d9%88/</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3547f32d-209e-4c3e-8686-35e670d8a57e/</t>
+        </is>
+      </c>
       <c r="R160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
@@ -12993,7 +13097,11 @@
           <t>https://royaldigi.ir/product/huawei-hg553/</t>
         </is>
       </c>
-      <c r="Q161" s="2" t="inlineStr"/>
+      <c r="Q161" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3c14cd83-c864-4316-9203-e3e3e6ca32b9/%D9%85%D9%88%D8%AF%D9%85-%D8%B1%D9%88%D8%AA%D8%B1-adsl-%D9%88%D8%AF%D8%A7%D9%81%D9%88%D9%86-%D9%85%D8%AF%D9%84-vodafone-hg553/</t>
+        </is>
+      </c>
       <c r="R161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
@@ -13071,7 +13179,11 @@
           <t>https://royaldigi.ir/product/naztech-nzt-tdx1000/</t>
         </is>
       </c>
-      <c r="Q162" s="2" t="inlineStr"/>
+      <c r="Q162" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3b1e326c-95ea-402a-9218-47209f98457c/</t>
+        </is>
+      </c>
       <c r="R162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
@@ -13146,10 +13258,14 @@
       </c>
       <c r="P163" s="2" t="inlineStr">
         <is>
-          <t>https://royaldigi.ir/?p=2564</t>
-        </is>
-      </c>
-      <c r="Q163" s="2" t="inlineStr"/>
+          <t>https://royaldigi.ir/product/huawei-b612s-25d/</t>
+        </is>
+      </c>
+      <c r="Q163" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/8233f2c5-5552-411a-b6e8-232a5118742d/</t>
+        </is>
+      </c>
       <c r="R163" s="2" t="inlineStr"/>
     </row>
     <row r="164">
@@ -13227,7 +13343,11 @@
           <t>https://royaldigi.ir/product/tp-link-xx230v/</t>
         </is>
       </c>
-      <c r="Q164" s="2" t="inlineStr"/>
+      <c r="Q164" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/23114068-d8a7-d985-d8af-d985-d981-db-8c-d8a8-d8b1-d986-d988-d8b1-db-8c-d8aa-db-8c-d9-be-d9-84-db-8c-d9-86-da-a9-d9-85-d8af-d9-84-xx230v-ax1800-d8af-d988-d8a8-d8a7-d9-86-d8af-wi-fi-6/</t>
+        </is>
+      </c>
       <c r="R164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
@@ -13305,7 +13425,11 @@
           <t>https://royaldigi.ir/product/mci-mc-i110/</t>
         </is>
       </c>
-      <c r="Q165" s="2" t="inlineStr"/>
+      <c r="Q165" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/653303c6-07f7-418e-a988-912f2750e386/</t>
+        </is>
+      </c>
       <c r="R165" s="2" t="inlineStr"/>
     </row>
     <row r="166">
@@ -13383,7 +13507,11 @@
           <t>https://royaldigi.ir/product/huawei-e5785-320/</t>
         </is>
       </c>
-      <c r="Q166" s="2" t="inlineStr"/>
+      <c r="Q166" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3b118b62-0943-41a4-96d2-8b4317f22557/</t>
+        </is>
+      </c>
       <c r="R166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
@@ -13461,7 +13589,11 @@
           <t>https://royaldigi.ir/product/huawei-e5785-320-stc/</t>
         </is>
       </c>
-      <c r="Q167" s="2" t="inlineStr"/>
+      <c r="Q167" s="2" t="inlineStr">
+        <is>
+          <t>https://torob.com/p/3b118b62-0943-41a4-96d2-8b4317f22557/</t>
+        </is>
+      </c>
       <c r="R167" s="2" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>